<commit_message>
Update on 12th NOv, 2025
</commit_message>
<xml_diff>
--- a/summary.xlsx
+++ b/summary.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
   <si>
     <t>Date</t>
   </si>
@@ -66,6 +66,30 @@
   </si>
   <si>
     <t>Knowledge Transfer to Iram and Viswaja regarding Alternate Authority implementation in ACE application.</t>
+  </si>
+  <si>
+    <t>Procedure and API creation for ACE application in HRMS.</t>
+  </si>
+  <si>
+    <t>Working on the editing, send to checker and corrsoponding status modification of a project. Also simultaniously creating preview of what has actually changed in the file.</t>
+  </si>
+  <si>
+    <t>Working on Creting batch when a batch has ended its life cycle.</t>
+  </si>
+  <si>
+    <t>Brainstorming with ACE team for creataion, consumption and implementation of newly ceated API of HRMS and also asked for An API from them to integrate in Dashboard PendingList.</t>
+  </si>
+  <si>
+    <t>"Send to Checker" and "Checker Action " batch wise has been completed.</t>
+  </si>
+  <si>
+    <t>What has changed by two different version as been developed. When Approver going to take action, a detailed view of changes have been showed to them.</t>
+  </si>
+  <si>
+    <t>Creating new batch on edit after approval,</t>
+  </si>
+  <si>
+    <t>Editing of the existing batch.</t>
   </si>
 </sst>
 </file>
@@ -393,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -501,25 +525,92 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2">
+        <v>45972</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2">
+        <v>45972</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2">
+        <v>45972</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2">
+        <v>45972</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2">
+        <v>45973</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2">
+        <v>45973</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2">
+        <v>45973</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>45973</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated on 18th November, 2025
</commit_message>
<xml_diff>
--- a/summary.xlsx
+++ b/summary.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
   <si>
     <t>Date</t>
   </si>
@@ -120,6 +120,33 @@
   </si>
   <si>
     <t>Provide help in ACE Enhancement also in Payroll Projection.</t>
+  </si>
+  <si>
+    <t>Provide solution for swipe mismatch change request, raised on 14-11-2025, by HR/Admin.</t>
+  </si>
+  <si>
+    <t>Modifying API as per recruirement from ACE.</t>
+  </si>
+  <si>
+    <t>Make provision to show Pending list of ACE application in HRMS dashboard pop-up window. API should be given by ACE team.</t>
+  </si>
+  <si>
+    <t>HRMS Branch marging, Procedure and table column transfer from Dev To Prod Server, and publishing of HRMS.</t>
+  </si>
+  <si>
+    <t>Fixing Redirection of ACE Application URL in HRMS.</t>
+  </si>
+  <si>
+    <t>Project Number Details and Post and Specialization under Project No modification in IPMS.</t>
+  </si>
+  <si>
+    <t>Fix Redirection of ACE Application URL in HRMS.</t>
+  </si>
+  <si>
+    <t>Fix issues after implementation of ACE pending list in HRMS, in production.</t>
+  </si>
+  <si>
+    <t>Created Logic of CO encashment for tax projection calculation and shared with Prachi.</t>
   </si>
 </sst>
 </file>
@@ -447,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -752,6 +779,116 @@
         <v>31</v>
       </c>
     </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>45978</v>
+      </c>
+      <c r="B33" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>45979</v>
+      </c>
+      <c r="B34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>45979</v>
+      </c>
+      <c r="B35" t="s">
+        <v>3</v>
+      </c>
+      <c r="C35" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>45979</v>
+      </c>
+      <c r="B36" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>45979</v>
+      </c>
+      <c r="B37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>